<commit_message>
Better Sort, missing gift
</commit_message>
<xml_diff>
--- a/Dary W20.xlsx
+++ b/Dary W20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RPG\Wilkolak\WoD-Gifts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC30059-F315-432C-9AE3-078B7559EEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38391143-C1E5-418D-BD16-6257D4FFB6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="6105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3717" uniqueCount="1112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3723" uniqueCount="1114">
   <si>
     <t>Rasa</t>
   </si>
@@ -3918,6 +3918,13 @@
   <si>
     <t>For many lupus-born, mankind’s technology proves difficult to grasp. This Gift allows a wolf in a bind to make use of human devices via the connection to the world afforded by Gnosis. Use of the Gift does not grant actual understanding of the device or system accessed; from an outsider’s perspective the technology simply cooperates with the Garou.
 System: The Garou rolls Wits + Primal-Urge (Difficulty 7) and spends a point of Gnosis. For the remainder of the scene, the Garou can substitute her Primal-Urge for rolls calling for Crafts, Drive, Etiquette, Firearms, and Larceny. With the expenditure of a point of Willpower, they can use Primal-Urge in place of Academics, Computer, Law, Science, and Technology rolls.</t>
+  </si>
+  <si>
+    <t>Trapper’s Bane</t>
+  </si>
+  <si>
+    <t>Dingoes throughout Australia, but especially near the dingo fence, face a constant threat from human traps — snares, steel traps, and poison. The dingoes have become adept at detecting these dangers and even disarming them. This Gift allows the werewolf to identify lures, traps, and even ambushes. Dingo spirits teach this Gift.
+System: The Storyteller rolls Perception + Primal Urge when the werewolf comes within (Gnosis × 5) yards of a trap’s trigger. The difficulty is 5 for the werewolf to detect simple snares, pits, and poisoned bait in the area. Identifying more technologically complex traps such as electrified objects and motion-activated traps is difficulty 6. Supernatural traps are difficulty 7. Additionally, whenever the werewolf approaches an ambush, the Storyteller rolls Perception + Primal Urge against difficulty 6 for the werewolf to recognize the ambush before it springs. The werewolf does not have to activate this Gift; it provides a “sixth sense” at all times.</t>
   </si>
 </sst>
 </file>
@@ -4238,7 +4245,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I619"/>
+  <dimension ref="A1:I620"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="22.42578125" customWidth="1"/>
@@ -4525,7 +4532,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
@@ -4750,7 +4757,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
@@ -4875,7 +4882,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>9</v>
       </c>
@@ -4925,7 +4932,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>9</v>
       </c>
@@ -5025,7 +5032,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>9</v>
       </c>
@@ -5150,7 +5157,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>9</v>
       </c>
@@ -5275,7 +5282,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>9</v>
       </c>
@@ -5400,7 +5407,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>9</v>
       </c>
@@ -5425,7 +5432,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>9</v>
       </c>
@@ -5475,7 +5482,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>9</v>
       </c>
@@ -5575,7 +5582,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>9</v>
       </c>
@@ -5825,7 +5832,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>9</v>
       </c>
@@ -5850,7 +5857,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>9</v>
       </c>
@@ -5875,7 +5882,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>9</v>
       </c>
@@ -5950,7 +5957,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>9</v>
       </c>
@@ -6025,7 +6032,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>9</v>
       </c>
@@ -6050,7 +6057,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>9</v>
       </c>
@@ -6275,7 +6282,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>9</v>
       </c>
@@ -6325,7 +6332,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>9</v>
       </c>
@@ -6425,7 +6432,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>9</v>
       </c>
@@ -6525,7 +6532,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>9</v>
       </c>
@@ -6625,7 +6632,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>9</v>
       </c>
@@ -6650,7 +6657,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>9</v>
       </c>
@@ -6775,7 +6782,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>9</v>
       </c>
@@ -6800,7 +6807,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>9</v>
       </c>
@@ -6975,7 +6982,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>9</v>
       </c>
@@ -7150,7 +7157,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>9</v>
       </c>
@@ -7300,7 +7307,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>9</v>
       </c>
@@ -7350,7 +7357,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>9</v>
       </c>
@@ -7375,7 +7382,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>9</v>
       </c>
@@ -7400,7 +7407,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>9</v>
       </c>
@@ -7425,7 +7432,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>9</v>
       </c>
@@ -7725,7 +7732,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>9</v>
       </c>
@@ -7825,7 +7832,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>9</v>
       </c>
@@ -7875,7 +7882,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>9</v>
       </c>
@@ -7900,7 +7907,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>9</v>
       </c>
@@ -7925,7 +7932,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>9</v>
       </c>
@@ -8050,7 +8057,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>9</v>
       </c>
@@ -8075,7 +8082,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>9</v>
       </c>
@@ -8225,7 +8232,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>9</v>
       </c>
@@ -8300,7 +8307,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>9</v>
       </c>
@@ -8325,7 +8332,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>9</v>
       </c>
@@ -8400,7 +8407,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>9</v>
       </c>
@@ -8475,7 +8482,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>9</v>
       </c>
@@ -8500,7 +8507,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>9</v>
       </c>
@@ -8575,7 +8582,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>9</v>
       </c>
@@ -8600,7 +8607,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>9</v>
       </c>
@@ -8700,7 +8707,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>9</v>
       </c>
@@ -8750,7 +8757,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>9</v>
       </c>
@@ -8775,7 +8782,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>9</v>
       </c>
@@ -8800,7 +8807,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>9</v>
       </c>
@@ -8900,7 +8907,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>9</v>
       </c>
@@ -8925,7 +8932,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>9</v>
       </c>
@@ -8950,7 +8957,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>9</v>
       </c>
@@ -8975,7 +8982,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>9</v>
       </c>
@@ -9100,7 +9107,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>9</v>
       </c>
@@ -9325,7 +9332,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>9</v>
       </c>
@@ -9350,7 +9357,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>9</v>
       </c>
@@ -9400,7 +9407,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>9</v>
       </c>
@@ -9500,7 +9507,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>9</v>
       </c>
@@ -9525,7 +9532,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>9</v>
       </c>
@@ -9600,7 +9607,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>9</v>
       </c>
@@ -9625,7 +9632,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>9</v>
       </c>
@@ -9675,7 +9682,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>9</v>
       </c>
@@ -9725,7 +9732,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>9</v>
       </c>
@@ -9775,7 +9782,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>9</v>
       </c>
@@ -9800,7 +9807,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>9</v>
       </c>
@@ -9825,7 +9832,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>9</v>
       </c>
@@ -9900,7 +9907,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>9</v>
       </c>
@@ -9925,7 +9932,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>9</v>
       </c>
@@ -9950,7 +9957,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>9</v>
       </c>
@@ -9975,7 +9982,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>9</v>
       </c>
@@ -10025,7 +10032,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>9</v>
       </c>
@@ -10075,7 +10082,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>9</v>
       </c>
@@ -10100,7 +10107,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>9</v>
       </c>
@@ -10250,7 +10257,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>9</v>
       </c>
@@ -10275,7 +10282,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>9</v>
       </c>
@@ -10300,7 +10307,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>9</v>
       </c>
@@ -10325,7 +10332,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>9</v>
       </c>
@@ -10400,7 +10407,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>9</v>
       </c>
@@ -10425,7 +10432,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>9</v>
       </c>
@@ -10475,7 +10482,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>9</v>
       </c>
@@ -10500,7 +10507,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>9</v>
       </c>
@@ -10550,7 +10557,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>9</v>
       </c>
@@ -10625,7 +10632,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>9</v>
       </c>
@@ -10650,7 +10657,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>9</v>
       </c>
@@ -10750,7 +10757,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>9</v>
       </c>
@@ -10800,7 +10807,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>9</v>
       </c>
@@ -10875,7 +10882,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>9</v>
       </c>
@@ -10925,7 +10932,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>9</v>
       </c>
@@ -10950,7 +10957,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>9</v>
       </c>
@@ -11075,7 +11082,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>9</v>
       </c>
@@ -11100,7 +11107,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>9</v>
       </c>
@@ -11125,7 +11132,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>9</v>
       </c>
@@ -11300,7 +11307,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>9</v>
       </c>
@@ -11325,7 +11332,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>9</v>
       </c>
@@ -11375,7 +11382,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
         <v>9</v>
       </c>
@@ -11450,7 +11457,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
         <v>9</v>
       </c>
@@ -11525,7 +11532,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>9</v>
       </c>
@@ -11550,7 +11557,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
         <v>9</v>
       </c>
@@ -11600,7 +11607,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
         <v>9</v>
       </c>
@@ -11775,7 +11782,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
         <v>9</v>
       </c>
@@ -11850,7 +11857,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>9</v>
       </c>
@@ -11875,7 +11882,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>9</v>
       </c>
@@ -11950,7 +11957,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>9</v>
       </c>
@@ -12000,7 +12007,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>9</v>
       </c>
@@ -12025,7 +12032,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>9</v>
       </c>
@@ -12125,7 +12132,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A316" s="1" t="s">
         <v>9</v>
       </c>
@@ -12175,7 +12182,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A318" s="1" t="s">
         <v>9</v>
       </c>
@@ -12200,7 +12207,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A319" s="1" t="s">
         <v>9</v>
       </c>
@@ -12300,7 +12307,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="323" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A323" s="1" t="s">
         <v>9</v>
       </c>
@@ -12375,7 +12382,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="326" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A326" s="1" t="s">
         <v>9</v>
       </c>
@@ -12425,7 +12432,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="328" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A328" s="1" t="s">
         <v>9</v>
       </c>
@@ -12500,7 +12507,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="331" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A331" s="1" t="s">
         <v>9</v>
       </c>
@@ -12525,7 +12532,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="332" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A332" s="1" t="s">
         <v>9</v>
       </c>
@@ -12550,7 +12557,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="333" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A333" s="1" t="s">
         <v>9</v>
       </c>
@@ -12600,7 +12607,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="335" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A335" s="1" t="s">
         <v>9</v>
       </c>
@@ -12650,7 +12657,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="337" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A337" s="1" t="s">
         <v>9</v>
       </c>
@@ -12675,7 +12682,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="338" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A338" s="1" t="s">
         <v>9</v>
       </c>
@@ -12700,7 +12707,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="339" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A339" s="1" t="s">
         <v>9</v>
       </c>
@@ -12725,7 +12732,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="340" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A340" s="1" t="s">
         <v>9</v>
       </c>
@@ -12775,7 +12782,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="342" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A342" s="1" t="s">
         <v>9</v>
       </c>
@@ -12800,7 +12807,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="343" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A343" s="1" t="s">
         <v>9</v>
       </c>
@@ -12850,7 +12857,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="345" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A345" s="1" t="s">
         <v>9</v>
       </c>
@@ -12900,7 +12907,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="347" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A347" s="1" t="s">
         <v>9</v>
       </c>
@@ -12925,7 +12932,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="348" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A348" s="1" t="s">
         <v>9</v>
       </c>
@@ -12975,7 +12982,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="350" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A350" s="1" t="s">
         <v>9</v>
       </c>
@@ -13000,7 +13007,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="351" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A351" s="1" t="s">
         <v>9</v>
       </c>
@@ -13025,7 +13032,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="352" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A352" s="1" t="s">
         <v>9</v>
       </c>
@@ -13075,7 +13082,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="354" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A354" s="1" t="s">
         <v>9</v>
       </c>
@@ -13150,7 +13157,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="357" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A357" s="1" t="s">
         <v>9</v>
       </c>
@@ -13175,7 +13182,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="358" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A358" s="1" t="s">
         <v>9</v>
       </c>
@@ -13200,7 +13207,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="359" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A359" s="1" t="s">
         <v>9</v>
       </c>
@@ -13225,7 +13232,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="360" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A360" s="1" t="s">
         <v>9</v>
       </c>
@@ -13250,7 +13257,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="361" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A361" s="1" t="s">
         <v>9</v>
       </c>
@@ -13275,7 +13282,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="362" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A362" s="1" t="s">
         <v>9</v>
       </c>
@@ -13325,7 +13332,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="364" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A364" s="1" t="s">
         <v>9</v>
       </c>
@@ -13350,7 +13357,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="365" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A365" s="1" t="s">
         <v>9</v>
       </c>
@@ -13425,7 +13432,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="368" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A368" s="1" t="s">
         <v>9</v>
       </c>
@@ -13450,7 +13457,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="369" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A369" s="1" t="s">
         <v>9</v>
       </c>
@@ -13500,7 +13507,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="371" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A371" s="1" t="s">
         <v>9</v>
       </c>
@@ -13525,7 +13532,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="372" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A372" s="1" t="s">
         <v>9</v>
       </c>
@@ -13650,7 +13657,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="377" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A377" s="1" t="s">
         <v>9</v>
       </c>
@@ -13700,7 +13707,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="379" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A379" s="1" t="s">
         <v>9</v>
       </c>
@@ -13725,7 +13732,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="380" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A380" s="1" t="s">
         <v>9</v>
       </c>
@@ -13750,7 +13757,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="381" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A381" s="1" t="s">
         <v>9</v>
       </c>
@@ -13775,7 +13782,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="382" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A382" s="1" t="s">
         <v>9</v>
       </c>
@@ -13800,7 +13807,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="383" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A383" s="1" t="s">
         <v>9</v>
       </c>
@@ -13900,7 +13907,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="387" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A387" s="1" t="s">
         <v>9</v>
       </c>
@@ -13950,7 +13957,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="389" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A389" s="1" t="s">
         <v>9</v>
       </c>
@@ -14025,7 +14032,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="392" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A392" s="1" t="s">
         <v>9</v>
       </c>
@@ -14050,7 +14057,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="393" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A393" s="1" t="s">
         <v>9</v>
       </c>
@@ -14175,7 +14182,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="398" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A398" s="1" t="s">
         <v>9</v>
       </c>
@@ -14200,7 +14207,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="399" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A399" s="1" t="s">
         <v>9</v>
       </c>
@@ -14250,7 +14257,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="401" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A401" s="1" t="s">
         <v>9</v>
       </c>
@@ -14375,7 +14382,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="406" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A406" s="1" t="s">
         <v>9</v>
       </c>
@@ -14525,7 +14532,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="412" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A412" s="1" t="s">
         <v>9</v>
       </c>
@@ -14550,7 +14557,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="413" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A413" s="1" t="s">
         <v>9</v>
       </c>
@@ -14600,7 +14607,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="415" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A415" s="1" t="s">
         <v>9</v>
       </c>
@@ -14650,7 +14657,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="417" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A417" s="1" t="s">
         <v>9</v>
       </c>
@@ -14675,7 +14682,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="418" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A418" s="1" t="s">
         <v>9</v>
       </c>
@@ -14750,7 +14757,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="421" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A421" s="1" t="s">
         <v>9</v>
       </c>
@@ -14800,7 +14807,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="423" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A423" s="1" t="s">
         <v>9</v>
       </c>
@@ -14850,7 +14857,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="425" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A425" s="1" t="s">
         <v>9</v>
       </c>
@@ -14925,7 +14932,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="428" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A428" s="1" t="s">
         <v>9</v>
       </c>
@@ -14950,7 +14957,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="429" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A429" s="1" t="s">
         <v>9</v>
       </c>
@@ -15025,7 +15032,7 @@
         <v>781</v>
       </c>
     </row>
-    <row r="432" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A432" s="1" t="s">
         <v>9</v>
       </c>
@@ -15100,7 +15107,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="435" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A435" s="1" t="s">
         <v>9</v>
       </c>
@@ -15125,7 +15132,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="436" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A436" s="1" t="s">
         <v>9</v>
       </c>
@@ -15225,7 +15232,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="440" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A440" s="1" t="s">
         <v>9</v>
       </c>
@@ -15250,7 +15257,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="441" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A441" s="1" t="s">
         <v>9</v>
       </c>
@@ -15275,7 +15282,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="442" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A442" s="1" t="s">
         <v>9</v>
       </c>
@@ -15300,7 +15307,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="443" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A443" s="1" t="s">
         <v>9</v>
       </c>
@@ -15375,7 +15382,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="446" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A446" s="1" t="s">
         <v>9</v>
       </c>
@@ -15425,7 +15432,7 @@
         <v>800</v>
       </c>
     </row>
-    <row r="448" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A448" s="1" t="s">
         <v>9</v>
       </c>
@@ -15475,7 +15482,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="450" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A450" s="1" t="s">
         <v>9</v>
       </c>
@@ -15500,7 +15507,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="451" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A451" s="1" t="s">
         <v>9</v>
       </c>
@@ -15525,7 +15532,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="452" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A452" s="1" t="s">
         <v>9</v>
       </c>
@@ -15575,7 +15582,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="454" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A454" s="1" t="s">
         <v>9</v>
       </c>
@@ -15600,7 +15607,7 @@
         <v>808</v>
       </c>
     </row>
-    <row r="455" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A455" s="1" t="s">
         <v>9</v>
       </c>
@@ -15675,7 +15682,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="458" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A458" s="1" t="s">
         <v>9</v>
       </c>
@@ -15700,7 +15707,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="459" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A459" s="1" t="s">
         <v>9</v>
       </c>
@@ -15775,7 +15782,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="462" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A462" s="1" t="s">
         <v>9</v>
       </c>
@@ -15800,7 +15807,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="463" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A463" s="1" t="s">
         <v>9</v>
       </c>
@@ -15825,7 +15832,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="464" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A464" s="1" t="s">
         <v>9</v>
       </c>
@@ -15850,7 +15857,7 @@
         <v>819</v>
       </c>
     </row>
-    <row r="465" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A465" s="1" t="s">
         <v>9</v>
       </c>
@@ -15875,7 +15882,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="466" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A466" s="1" t="s">
         <v>9</v>
       </c>
@@ -15900,7 +15907,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="467" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A467" s="1" t="s">
         <v>9</v>
       </c>
@@ -15975,7 +15982,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="470" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A470" s="1" t="s">
         <v>9</v>
       </c>
@@ -16000,7 +16007,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="471" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A471" s="1" t="s">
         <v>9</v>
       </c>
@@ -16075,7 +16082,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="474" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A474" s="1" t="s">
         <v>9</v>
       </c>
@@ -16125,7 +16132,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="476" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A476" s="1" t="s">
         <v>9</v>
       </c>
@@ -16150,7 +16157,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="477" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A477" s="1" t="s">
         <v>9</v>
       </c>
@@ -16175,7 +16182,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="478" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A478" s="1" t="s">
         <v>9</v>
       </c>
@@ -16200,7 +16207,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="479" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A479" s="1" t="s">
         <v>9</v>
       </c>
@@ -16500,7 +16507,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="491" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A491" s="1" t="s">
         <v>9</v>
       </c>
@@ -16525,7 +16532,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="492" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A492" s="1" t="s">
         <v>9</v>
       </c>
@@ -16575,7 +16582,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="494" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A494" s="1" t="s">
         <v>9</v>
       </c>
@@ -16650,7 +16657,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="497" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A497" s="1" t="s">
         <v>9</v>
       </c>
@@ -16700,7 +16707,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="499" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A499" s="1" t="s">
         <v>9</v>
       </c>
@@ -16775,7 +16782,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="502" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A502" s="1" t="s">
         <v>9</v>
       </c>
@@ -17050,7 +17057,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="513" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="513" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A513" s="1" t="s">
         <v>9</v>
       </c>
@@ -17150,7 +17157,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="517" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="517" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A517" s="1" t="s">
         <v>9</v>
       </c>
@@ -17300,7 +17307,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="523" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="523" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A523" s="1" t="s">
         <v>9</v>
       </c>
@@ -17350,7 +17357,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="525" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="525" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A525" s="1" t="s">
         <v>9</v>
       </c>
@@ -17400,7 +17407,7 @@
         <v>930</v>
       </c>
     </row>
-    <row r="527" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="527" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A527" s="1" t="s">
         <v>9</v>
       </c>
@@ -17450,7 +17457,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="529" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="529" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A529" s="1" t="s">
         <v>9</v>
       </c>
@@ -17500,7 +17507,7 @@
         <v>937</v>
       </c>
     </row>
-    <row r="531" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="531" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A531" s="1" t="s">
         <v>9</v>
       </c>
@@ -17575,7 +17582,7 @@
         <v>942</v>
       </c>
     </row>
-    <row r="534" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="534" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A534" s="1" t="s">
         <v>9</v>
       </c>
@@ -19723,6 +19730,31 @@
       <c r="H619" s="1"/>
       <c r="I619" s="1" t="s">
         <v>1111</v>
+      </c>
+    </row>
+    <row r="620" spans="1:9" ht="120" x14ac:dyDescent="0.25">
+      <c r="A620" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B620" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C620" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="D620" s="1">
+        <v>2</v>
+      </c>
+      <c r="E620" s="1"/>
+      <c r="F620" t="s">
+        <v>1112</v>
+      </c>
+      <c r="G620" s="1" t="s">
+        <v>949</v>
+      </c>
+      <c r="H620" s="1"/>
+      <c r="I620" s="1" t="s">
+        <v>1113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>